<commit_message>
Fix GC regression tests and Memgraph expectations for QA filters
</commit_message>
<xml_diff>
--- a/InputFiles/GC/TC05_GC_phs003432_Sex-Female_PrimDiag_NotReported_FileType-RDS.xlsx
+++ b/InputFiles/GC/TC05_GC_phs003432_Sex-Female_PrimDiag_NotReported_FileType-RDS.xlsx
@@ -506,12 +506,13 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATCH (d:diagnosis)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+          <t>MATCH (d:diagnosis)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
 MATCH (f:file)-[:of_participant]-&gt;(p)
 WHERE s.phs_accession = "phs003432"
   AND p.sex = "Female"
   AND d.primary_diagnosis = "Not Reported"
   AND toLower(f.file_type) = toLower("RDS")
+  AND p.dbGaP_subject_id IS NOT NULL AND trim(p.dbGaP_subject_id) &lt;&gt; ""
 WITH DISTINCT p, s
 OPTIONAL MATCH (samp_all:sample)-[:of_participant]-&gt;(p)
 WITH p, s, samp_all
@@ -525,30 +526,40 @@
   END AS samples
 RETURN
   p.participant_id AS participant_id,
-  s.study_name AS study_name,
+  s.study_acronym AS study_name,
   s.phs_accession AS accession,
   p.sex AS sex,
-  samples
+  samples AS samples
 ORDER BY p.participant_id ASC
-LIMIT 100
-</t>
+LIMIT 100</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATCH (d:diagnosis)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
-MATCH (f:file)-[:of_participant]-&gt;(p)
+          <t>MATCH (s:study)
 WHERE s.phs_accession = "phs003432"
-  AND p.sex = "Female"
+OPTIONAL MATCH (d:diagnosis)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s)
+WHERE p.sex = "Female"
   AND d.primary_diagnosis = "Not Reported"
-  AND toLower(f.file_type) = toLower("RDS")
-OPTIONAL MATCH (f)-[:from_sample]-&gt;(samp:sample)
-RETURN
-  count(DISTINCT s) AS Studies,
-  count(DISTINCT p) AS Participants,
-  count(DISTINCT samp) AS Samples,
-  count(DISTINCT f) AS Files
-</t>
+  AND p.dbGaP_subject_id IS NOT NULL AND trim(p.dbGaP_subject_id) &lt;&gt; ""
+OPTIONAL MATCH (f_p:file)-[:of_participant]-&gt;(p)
+WHERE toLower(f_p.file_type) = toLower("RDS")
+OPTIONAL MATCH (f_p)-[:from_sample]-&gt;(samp:sample)-[:of_participant]-&gt;(p)
+WITH s, collect(DISTINCT p) AS parts, collect(DISTINCT samp) AS samps
+MATCH (f:file)-[:of_study]-&gt;(s)
+WHERE toLower(f.file_type) = toLower("RDS")
+  AND EXISTS {
+    MATCH (f)-[:of_participant]-&gt;(p2:participant)
+    WHERE p2.sex = "Female"
+      AND EXISTS {
+        MATCH (d2:diagnosis)-[:of_participant]-&gt;(p2)
+        WHERE d2.primary_diagnosis = "Not Reported"
+      }
+  }
+RETURN count(DISTINCT s) AS Studies,
+  size([x IN parts WHERE x IS NOT NULL]) AS Participants,
+  size([x IN samps WHERE x IS NOT NULL]) AS Samples,
+  count(DISTINCT f) AS Files</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -570,12 +581,13 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATCH (d:diagnosis)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+          <t>MATCH (d:diagnosis)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
 MATCH (f:file)-[:from_sample]-&gt;(samp:sample)-[:of_participant]-&gt;(p)
 WHERE s.phs_accession = "phs003432"
   AND p.sex = "Female"
   AND d.primary_diagnosis = "Not Reported"
   AND toLower(f.file_type) = toLower("RDS")
+  AND p.dbGaP_subject_id IS NOT NULL AND trim(p.dbGaP_subject_id) &lt;&gt; ""
 RETURN DISTINCT
   s.study_acronym AS study_name,
   s.phs_accession AS accession,
@@ -583,8 +595,7 @@
   COALESCE(samp.sample_name, samp.sample_id) AS sample_name,
   COALESCE(samp.Organization_Name, "Not specified in data") AS organization_name
 ORDER BY samp.sample_id ASC
-LIMIT 100
-</t>
+LIMIT 100</t>
         </is>
       </c>
       <c r="C3" s="2" t="n"/>
@@ -597,23 +608,36 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATCH (d:diagnosis)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
-MATCH (f:file)-[:of_participant]-&gt;(p)
+          <t>MATCH (f:file)-[:of_study]-&gt;(s:study)
 WHERE s.phs_accession = "phs003432"
-  AND p.sex = "Female"
-  AND d.primary_diagnosis = "Not Reported"
   AND toLower(f.file_type) = toLower("RDS")
-OPTIONAL MATCH (f)-[:from_sample]-&gt;(samp:sample)
-RETURN DISTINCT
+  AND EXISTS {
+    MATCH (f)-[:of_participant]-&gt;(p:participant)
+    WHERE p.sex = "Female"
+      AND EXISTS {
+        MATCH (d:diagnosis)-[:of_participant]-&gt;(p)
+        WHERE d.primary_diagnosis = "Not Reported"
+      }
+  }
+WITH DISTINCT s, f
+OPTIONAL MATCH (f)-[:from_sample]-&gt;(all_samp:sample)
+WITH s, f, all_samp
+ORDER BY all_samp.sample_id ASC
+WITH s, f, [x IN collect(DISTINCT all_samp.sample_id) WHERE x IS NOT NULL] AS sample_ids
+RETURN
   s.study_name AS study_name,
   s.phs_accession AS accession,
   f.file_name AS file_name,
   f.file_id AS file_id,
   f.file_type AS file_type,
-  COALESCE(samp.sample_id, "Not Applicable") AS sample_id
+  CASE
+    WHEN size(sample_ids) = 0 THEN "Not Applicable"
+    WHEN size(sample_ids) &gt; 5
+    THEN reduce(acc = "", id IN sample_ids[0..5] | CASE WHEN acc = "" THEN id ELSE acc + ", " + id END) + ", ..."
+    ELSE reduce(acc = "", id IN sample_ids | CASE WHEN acc = "" THEN id ELSE acc + ", " + id END)
+  END AS sample_id
 ORDER BY f.file_name ASC
-LIMIT 100
-</t>
+LIMIT 100</t>
         </is>
       </c>
       <c r="C4" s="2" t="n"/>

</xml_diff>